<commit_message>
update new note and feature
</commit_message>
<xml_diff>
--- a/data/ROSA/Testing_Module.xlsx
+++ b/data/ROSA/Testing_Module.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10909"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WTK_TestPlaner\data\ROSA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/victor/Desktop/TestPlaner/WTK_TestPlaner/data/ROSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{646BB588-82C0-4688-B9E1-75A1B35934E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BBC27E3-4D63-AF44-890D-D059181812D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-380" yWindow="660" windowWidth="30240" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,15 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="32">
   <si>
     <t>TestingMoudleID</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -130,16 +127,14 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>MODULE_ID_Z</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>MODULE_ID_XY</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>FUNC_UFIT_ORV3</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ModuleID</t>
+  </si>
+  <si>
+    <t>MODULE_ID</t>
   </si>
 </sst>
 </file>
@@ -150,13 +145,13 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="新細明體"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="新細明體"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="136"/>
       <scheme val="minor"/>
@@ -198,7 +193,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="一般" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -476,222 +471,258 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.125" customWidth="1"/>
-    <col min="2" max="2" width="22.5" customWidth="1"/>
-    <col min="3" max="3" width="24.25" customWidth="1"/>
-    <col min="4" max="4" width="24.75" customWidth="1"/>
-    <col min="5" max="5" width="26.875" customWidth="1"/>
-    <col min="6" max="6" width="25.625" customWidth="1"/>
-    <col min="7" max="7" width="22.625" customWidth="1"/>
-    <col min="8" max="8" width="18.625" customWidth="1"/>
-    <col min="9" max="9" width="18.125" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="2" max="2" width="24.1640625" customWidth="1"/>
+    <col min="3" max="3" width="22.5" customWidth="1"/>
+    <col min="4" max="4" width="24.1640625" customWidth="1"/>
+    <col min="5" max="5" width="24.6640625" customWidth="1"/>
+    <col min="6" max="6" width="26.83203125" customWidth="1"/>
+    <col min="7" max="7" width="25.6640625" customWidth="1"/>
+    <col min="8" max="8" width="22.6640625" customWidth="1"/>
+    <col min="9" max="9" width="18.6640625" customWidth="1"/>
+    <col min="10" max="10" width="18.1640625" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="1" t="s">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>14</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="I3" s="1" t="s">
+      <c r="F3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>14</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="1" t="s">
+      <c r="C7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="1" t="s">
+      <c r="C8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="1" t="s">
+      <c r="C9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="1" t="s">
+      <c r="C10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" s="1" t="s">
+      <c r="C11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E11" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="G11" s="1"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C11" s="1" t="s">
+      <c r="C12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F11" s="1"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>14</v>
-      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J11">
-    <sortCondition ref="A2:A11"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:K11">
+    <sortCondition ref="B2:B11"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add test plan combinaiton matrix
</commit_message>
<xml_diff>
--- a/data/ROSA/Testing_Module.xlsx
+++ b/data/ROSA/Testing_Module.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/victor/Desktop/TestPlaner/WTK_TestPlaner/data/ROSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BBC27E3-4D63-AF44-890D-D059181812D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41403C22-B0B0-6F4A-AAB1-5BF4929F3EF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-380" yWindow="660" windowWidth="30240" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15100" yWindow="660" windowWidth="15140" windowHeight="17800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,16 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="35">
   <si>
     <t>TestingMoudleID</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve">Testing Item Sequence </t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>NONOP_L10</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -123,10 +119,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>MODULE_ID</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>FUNC_UFIT_ORV3</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -134,7 +126,22 @@
     <t>ModuleID</t>
   </si>
   <si>
-    <t>MODULE_ID</t>
+    <t>PARAM_1</t>
+  </si>
+  <si>
+    <t>PARAM_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Testing Item ID Sequence </t>
+  </si>
+  <si>
+    <t>2 system</t>
+  </si>
+  <si>
+    <t>3 system</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 system </t>
   </si>
 </sst>
 </file>
@@ -157,7 +164,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -167,6 +174,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -183,12 +196,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -471,7 +487,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="24.1640625" customWidth="1"/>
@@ -486,238 +502,263 @@
     <col min="11" max="11" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="E3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>14</v>
+        <v>7</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>29</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="G11" s="1"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>